<commit_message>
Updated BOM to remove Raspberry PI. Added step down regulator CAD
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="48">
   <si>
     <t>Category</t>
   </si>
@@ -109,22 +109,19 @@
     <t>5.2V</t>
   </si>
   <si>
-    <t>Raspberry Pi 5 (16GB)</t>
-  </si>
-  <si>
-    <t>5.0V</t>
-  </si>
-  <si>
-    <t>Raspberry Pi AI Camera</t>
-  </si>
-  <si>
-    <t>5.0V / 12V</t>
+    <t>Holybro SiK Telemetry Radio V3</t>
+  </si>
+  <si>
+    <t>5V</t>
   </si>
   <si>
     <t>Regulators</t>
   </si>
   <si>
     <t>10A High Voltage UBEC</t>
+  </si>
+  <si>
+    <t>Up to 6S</t>
   </si>
   <si>
     <t>Pololu 5V 9A Step-Down Voltage Regulator</t>
@@ -177,7 +174,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -188,6 +185,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9EAD3"/>
         <bgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -209,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -220,6 +223,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -512,6 +516,7 @@
       <c r="G3" s="1">
         <v>43.99</v>
       </c>
+      <c r="H3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
@@ -535,6 +540,7 @@
       <c r="G4" s="1">
         <v>260.0</v>
       </c>
+      <c r="H4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
@@ -558,6 +564,7 @@
       <c r="G5" s="1">
         <v>170.0</v>
       </c>
+      <c r="H5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
@@ -581,6 +588,7 @@
       <c r="G6" s="1">
         <v>180.0</v>
       </c>
+      <c r="H6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
@@ -605,6 +613,7 @@
         <f>84.99*2</f>
         <v>169.98</v>
       </c>
+      <c r="H7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
@@ -629,6 +638,7 @@
         <f>41.99 *4</f>
         <v>167.96</v>
       </c>
+      <c r="H8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
@@ -653,6 +663,7 @@
         <f>14.99*2</f>
         <v>29.98</v>
       </c>
+      <c r="H9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
@@ -677,6 +688,7 @@
         <f>5.99*2</f>
         <v>11.98</v>
       </c>
+      <c r="H10" s="4"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
@@ -701,6 +713,7 @@
         <f>13.99*2</f>
         <v>27.98</v>
       </c>
+      <c r="H11" s="4"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
@@ -724,6 +737,7 @@
       <c r="G12" s="1">
         <v>165.99</v>
       </c>
+      <c r="H12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
@@ -736,44 +750,46 @@
         <v>1.0</v>
       </c>
       <c r="D13" s="1">
-        <v>97.0</v>
+        <v>67.0</v>
       </c>
       <c r="E13" s="1">
-        <v>97.0</v>
+        <v>67.0</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>33</v>
       </c>
       <c r="G13" s="1">
-        <v>338.39</v>
-      </c>
+        <v>58.99</v>
+      </c>
+      <c r="H13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C14" s="1">
         <v>1.0</v>
       </c>
       <c r="D14" s="1">
-        <v>18.0</v>
+        <v>14.0</v>
       </c>
       <c r="E14" s="1">
-        <v>18.0</v>
+        <v>14.0</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G14" s="1">
-        <v>77.99</v>
-      </c>
+        <v>38.99</v>
+      </c>
+      <c r="H14" s="4"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>37</v>
@@ -782,53 +798,45 @@
         <v>1.0</v>
       </c>
       <c r="D15" s="1">
-        <v>34.0</v>
+        <v>10.0</v>
       </c>
       <c r="E15" s="1">
-        <v>34.0</v>
+        <v>10.0</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="G15" s="1">
-        <v>38.99</v>
-      </c>
+        <v>36.82</v>
+      </c>
+      <c r="H15" s="2"/>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="D16" s="1">
-        <v>10.0</v>
-      </c>
-      <c r="E16" s="1">
-        <v>10.0</v>
-      </c>
-      <c r="F16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="1">
-        <v>36.82</v>
+      <c r="E16" s="5">
+        <f>SUM(E2:E15)</f>
+        <v>1371.8</v>
       </c>
     </row>
     <row r="17">
-      <c r="D17" s="1" t="s">
+      <c r="A17" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="4">
-        <f>SUM(E2:E16)</f>
-        <v>1439.8</v>
+      <c r="B17" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="G17" s="1">
+        <v>379.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>42</v>
@@ -837,12 +845,12 @@
         <v>1.0</v>
       </c>
       <c r="G18" s="1">
-        <v>379.0</v>
+        <v>29.99</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>43</v>
@@ -851,59 +859,45 @@
         <v>1.0</v>
       </c>
       <c r="G19" s="1">
-        <v>29.99</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C20" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="G20" s="1">
-        <v>10.0</v>
+        <v>4.0</v>
+      </c>
+      <c r="G20" s="3">
+        <f>22.99*4</f>
+        <v>91.96</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C21" s="1">
-        <v>4.0</v>
-      </c>
-      <c r="G21" s="3">
-        <f>22.99*4</f>
-        <v>91.96</v>
+        <v>1.0</v>
+      </c>
+      <c r="G21" s="1">
+        <v>20.0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="G22" s="1">
-        <v>20.0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="F23" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G23" s="5">
-        <f>sum(G2:G22)</f>
-        <v>2400.99</v>
+      <c r="G22" s="6">
+        <f>sum(G2:G21)</f>
+        <v>2043.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added materials and image to BOM
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -1,17 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Director\Downloads\VFS\Summer 26\VTOL Flying Wing project\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0759BCA-3F2B-48AF-94B9-E136FE0B40C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="27634" windowHeight="17349" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="page 1" sheetId="1" r:id="rId5"/>
+    <sheet name="page 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
   <si>
     <t>Category</t>
   </si>
@@ -155,20 +177,24 @@
   </si>
   <si>
     <t>Total price</t>
+  </si>
+  <si>
+    <t>Filament</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -179,7 +205,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -207,41 +233,92 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>118753</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>67747</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0AF60F2D-DBD9-474A-BF56-F93019158AED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9856520" y="197923"/>
+          <a:ext cx="5462649" cy="3630344"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -431,20 +508,23 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultColWidth="12.61328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="38.63"/>
+    <col min="2" max="2" width="38.61328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -470,7 +550,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -478,13 +558,13 @@
         <v>9</v>
       </c>
       <c r="C2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1">
-        <v>690.0</v>
+        <v>690</v>
       </c>
       <c r="E2" s="1">
-        <v>690.0</v>
+        <v>690</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -494,7 +574,7 @@
       </c>
       <c r="H2" s="2"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -502,7 +582,7 @@
         <v>11</v>
       </c>
       <c r="C3" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D3" s="1">
         <v>43.8</v>
@@ -518,7 +598,7 @@
       </c>
       <c r="H3" s="2"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -526,23 +606,23 @@
         <v>14</v>
       </c>
       <c r="C4" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="1">
-        <v>190.0</v>
+        <v>190</v>
       </c>
       <c r="E4" s="1">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G4" s="1">
-        <v>260.0</v>
+        <v>260</v>
       </c>
       <c r="H4" s="2"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -550,23 +630,23 @@
         <v>16</v>
       </c>
       <c r="C5" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D5" s="1">
-        <v>250.0</v>
+        <v>250</v>
       </c>
       <c r="E5" s="1">
-        <v>35.0</v>
+        <v>35</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="1">
-        <v>170.0</v>
+        <v>170</v>
       </c>
       <c r="H5" s="2"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -574,23 +654,23 @@
         <v>18</v>
       </c>
       <c r="C6" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1">
-        <v>55.0</v>
+        <v>55</v>
       </c>
       <c r="E6" s="1">
-        <v>55.0</v>
+        <v>55</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G6" s="1">
-        <v>180.0</v>
+        <v>180</v>
       </c>
       <c r="H6" s="2"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
@@ -598,7 +678,7 @@
         <v>20</v>
       </c>
       <c r="C7" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D7" s="1">
         <v>52.4</v>
@@ -615,7 +695,7 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
@@ -623,24 +703,24 @@
         <v>22</v>
       </c>
       <c r="C8" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="D8" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="E8" s="1">
-        <v>36.0</v>
+        <v>36</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="1">
         <f>41.99 *4</f>
         <v>167.96</v>
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -648,7 +728,7 @@
         <v>25</v>
       </c>
       <c r="C9" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D9" s="1">
         <v>9.6</v>
@@ -659,13 +739,13 @@
       <c r="F9" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="1">
         <f>14.99*2</f>
         <v>29.98</v>
       </c>
       <c r="H9" s="2"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>24</v>
       </c>
@@ -673,7 +753,7 @@
         <v>27</v>
       </c>
       <c r="C10" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D10" s="1">
         <v>1.2</v>
@@ -684,13 +764,13 @@
       <c r="F10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="1">
         <f>5.99*2</f>
         <v>11.98</v>
       </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11">
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
@@ -698,13 +778,13 @@
         <v>28</v>
       </c>
       <c r="C11" s="1">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="D11" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="E11" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>26</v>
@@ -713,9 +793,9 @@
         <f>13.99*2</f>
         <v>27.98</v>
       </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12">
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>29</v>
       </c>
@@ -723,7 +803,7 @@
         <v>30</v>
       </c>
       <c r="C12" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D12" s="1">
         <v>34.6</v>
@@ -739,7 +819,7 @@
       </c>
       <c r="H12" s="2"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>29</v>
       </c>
@@ -747,13 +827,13 @@
         <v>32</v>
       </c>
       <c r="C13" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="1">
-        <v>67.0</v>
+        <v>67</v>
       </c>
       <c r="E13" s="1">
-        <v>67.0</v>
+        <v>67</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>33</v>
@@ -763,7 +843,7 @@
       </c>
       <c r="H13" s="2"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>34</v>
       </c>
@@ -771,13 +851,13 @@
         <v>35</v>
       </c>
       <c r="C14" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="E14" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>36</v>
@@ -785,9 +865,9 @@
       <c r="G14" s="1">
         <v>38.99</v>
       </c>
-      <c r="H14" s="4"/>
-    </row>
-    <row r="15">
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
@@ -795,13 +875,13 @@
         <v>37</v>
       </c>
       <c r="C15" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="E15" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>38</v>
@@ -811,16 +891,16 @@
       </c>
       <c r="H15" s="2"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D16" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="4">
         <f>SUM(E2:E15)</f>
         <v>1371.8</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>40</v>
       </c>
@@ -828,13 +908,13 @@
         <v>41</v>
       </c>
       <c r="C17" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="1">
-        <v>379.0</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>40</v>
       </c>
@@ -842,13 +922,13 @@
         <v>42</v>
       </c>
       <c r="C18" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="1">
         <v>29.99</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
@@ -856,51 +936,72 @@
         <v>43</v>
       </c>
       <c r="C19" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="1">
-        <v>10.0</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="1">
+        <v>1</v>
+      </c>
+      <c r="G20" s="1">
+        <v>21.99</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="1">
-        <v>4.0</v>
-      </c>
-      <c r="G20" s="3">
+      <c r="C22" s="1">
+        <v>4</v>
+      </c>
+      <c r="G22" s="1">
         <f>22.99*4</f>
         <v>91.96</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="s">
+    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="1">
-        <v>1.0</v>
-      </c>
-      <c r="G21" s="1">
-        <v>20.0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="F22" s="1" t="s">
+      <c r="C23" s="1">
+        <v>1</v>
+      </c>
+      <c r="G23" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F24" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="G22" s="6">
-        <f>sum(G2:G21)</f>
-        <v>2043.6</v>
+      <c r="G24" s="5">
+        <f>SUM(G2:G23)</f>
+        <v>2065.59</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>